<commit_message>
Finalizaçao da respostas automaticas
</commit_message>
<xml_diff>
--- a/Avaliacao_2/Planilha_Mestra.xlsx
+++ b/Avaliacao_2/Planilha_Mestra.xlsx
@@ -522,15 +522,13 @@
           <t>Rua das Acacias, 245 - Apto 302, Parque das Laranjeiras, Manaus - AM, 69000-000</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
       <c r="H2" s="6" t="n">
-        <v>46245.72116934536</v>
+        <v>46245.72116934028</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -557,15 +555,13 @@
           <t>Rua das Palmeiras, 120 - Flores, Flores, Manaus - AM, 69058-000</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
       <c r="H3" s="6" t="n">
-        <v>46245.72116941064</v>
+        <v>46245.72116940972</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -600,7 +596,7 @@
         </is>
       </c>
       <c r="H4" s="6" t="n">
-        <v>46245.72116948877</v>
+        <v>46245.72683256326</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>

</xml_diff>